<commit_message>
fix: MRSH column alignment matched to AON layout
</commit_message>
<xml_diff>
--- a/output/comp_sheet_updated.xlsx
+++ b/output/comp_sheet_updated.xlsx
@@ -10923,65 +10923,59 @@
         </is>
       </c>
       <c r="C57" s="55">
-        <f>_xll.BDP("MMC US Equity","CUR_MKT_CAP")/1000000000</f>
+        <f>BDP("MRSH US Equity","CUR_MKT_CAP")/1000000000</f>
         <v/>
       </c>
       <c r="D57" s="56">
-        <f>_xll.BDP("MRSH US Equity","CUR_MKT_CAP")/1000000000</f>
+        <f>BDP("MRSH US Equity","PX_LAST")</f>
         <v/>
       </c>
       <c r="E57" s="57">
-        <f>_xll.BDP("MRSH US Equity","PX_LAST")</f>
+        <f>IF(BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,$D$57/BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
         <v/>
       </c>
       <c r="F57" s="57">
-        <f>IF(_xll.BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,$E$57/_xll.BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
+        <f>IF(BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")&lt;&gt;0,$D$57/BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y"),"")</f>
         <v/>
       </c>
       <c r="G57" s="57">
-        <f>IF(_xll.BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")&lt;&gt;0,$E$57/_xll.BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y"),"")</f>
+        <f>IF(BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&lt;&gt;0,$D$57/BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y"),"")</f>
         <v/>
       </c>
       <c r="H57" s="58">
-        <f>IF(_xll.BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&lt;&gt;0,$E$57/_xll.BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y"),"")</f>
+        <f>BDP("MRSH US Equity","NET_DEBT_TO_EBITDA")</f>
         <v/>
       </c>
       <c r="I57" s="55">
-        <f>_xll.BDP("MRSH US Equity","NET_DEBT_TO_EBITDA")</f>
+        <f>BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")/1000</f>
         <v/>
       </c>
       <c r="J57" s="59">
-        <f>_xll.BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")/1000</f>
+        <f>IF(BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")/BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
         <v/>
       </c>
       <c r="K57" s="59">
-        <f>IF(_xll.BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,_xll.BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")/_xll.BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
+        <f>BDP("MRSH US Equity","RETURN_ON_INV_CAPITAL")/100</f>
         <v/>
       </c>
       <c r="L57" s="59">
-        <f>_xll.BDP("MRSH US Equity","RETURN_ON_INV_CAPITAL")/100</f>
+        <f>IF(AND(BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")/BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
         <v/>
       </c>
       <c r="M57" s="55">
-        <f>IF(AND(_xll.BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,_xll.BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(_xll.BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")/_xll.BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
+        <f>IF(AND(BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")/BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
         <v/>
       </c>
       <c r="N57" s="59">
-        <f>IF(AND(_xll.BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,_xll.BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(_xll.BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")/_xll.BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="O57" s="60">
-        <f>IF(AND(_xll.BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,_xll.BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(_xll.BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")/_xll.BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
+        <f>IF(AND(BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")/BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
+        <v/>
+      </c>
+      <c r="O57" s="60" t="n"/>
       <c r="P57" s="59">
-        <f>_xll.BDP("MMC US Equity","CHG_PCT_YTD")/100</f>
-        <v/>
-      </c>
-      <c r="Q57" s="60">
-        <f>_xll.BDP("MRSH US Equity","CHG_PCT_YTD")/100</f>
-        <v/>
-      </c>
+        <f>BDP("MRSH US Equity","CHG_PCT_YTD")/100</f>
+        <v/>
+      </c>
+      <c r="Q57" s="60" t="n"/>
       <c r="R57" s="1" t="n"/>
       <c r="S57" s="40">
         <f>IF(AND(E57&lt;&gt;"",N57&lt;&gt;"",N57&lt;&gt;0),E57/(N57*100),"")</f>
@@ -10998,115 +10992,115 @@
       <c r="X57" s="1" t="n"/>
       <c r="Y57" s="1" t="n"/>
       <c r="Z57" s="1" t="n"/>
-      <c r="AA57" s="1" t="n"/>
+      <c r="AA57" s="60">
+        <f>BDP("MRSH US Equity","TRAIL_12M_OPER_INC")</f>
+        <v/>
+      </c>
       <c r="AB57" s="55">
-        <f>_xll.BDP("MRSH US Equity","TRAIL_12M_OPER_INC")</f>
+        <f>BDP("MRSH US Equity","SHORT_AND_LONG_TERM_DEBT")</f>
         <v/>
       </c>
       <c r="AC57" s="55">
-        <f>_xll.BDP("MRSH US Equity","SHORT_AND_LONG_TERM_DEBT")</f>
+        <f>BDP("MRSH US Equity","TOTAL_EQUITY")</f>
         <v/>
       </c>
       <c r="AD57" s="55">
-        <f>_xll.BDP("MRSH US Equity","TOTAL_EQUITY")</f>
+        <f>BDP("MRSH US Equity","BS_CASH_NEAR_CASH_ITEM")</f>
         <v/>
       </c>
       <c r="AE57" s="55">
-        <f>_xll.BDP("MRSH US Equity","BS_CASH_NEAR_CASH_ITEM")</f>
+        <f>BDP("MRSH US Equity","BS_LT_INVEST")</f>
         <v/>
       </c>
       <c r="AF57" s="55">
-        <f>_xll.BDP("MRSH US Equity","BS_LT_INVEST")</f>
-        <v/>
-      </c>
-      <c r="AG57" s="4">
-        <f>AC57+AD57</f>
-        <v/>
-      </c>
-      <c r="AH57" s="59">
-        <f>_xll.BDP("MRSH US Equity","RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
-      <c r="AI57" s="1" t="n"/>
+        <f>AB57+AC57</f>
+        <v/>
+      </c>
+      <c r="AG57" s="55">
+        <f>BDP("MRSH US Equity","RETURN_ON_INV_CAPITAL")/100</f>
+        <v/>
+      </c>
+      <c r="AH57" s="59" t="n"/>
+      <c r="AI57" s="60">
+        <f>BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","24Y")</f>
+        <v/>
+      </c>
       <c r="AJ57" s="55">
-        <f>_xll.BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","24Y")</f>
+        <f>BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")</f>
         <v/>
       </c>
       <c r="AK57" s="55">
-        <f>_xll.BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")</f>
+        <f>BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")</f>
         <v/>
       </c>
       <c r="AL57" s="55">
-        <f>_xll.BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")</f>
+        <f>BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")</f>
         <v/>
       </c>
       <c r="AM57" s="55">
-        <f>_xll.BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AN57" s="55">
-        <f>_xll.BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
-      <c r="AO57" s="1" t="n"/>
+        <f>BDP("MRSH US Equity","BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")</f>
+        <v/>
+      </c>
+      <c r="AN57" s="55" t="n"/>
+      <c r="AO57" s="60">
+        <f>BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","24Y")</f>
+        <v/>
+      </c>
       <c r="AP57" s="55">
-        <f>_xll.BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","24Y")</f>
+        <f>BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")</f>
         <v/>
       </c>
       <c r="AQ57" s="55">
-        <f>_xll.BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")</f>
+        <f>BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")</f>
         <v/>
       </c>
       <c r="AR57" s="55">
-        <f>_xll.BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")</f>
+        <f>BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","27Y")</f>
         <v/>
       </c>
       <c r="AS57" s="55">
-        <f>_xll.BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AT57" s="55">
-        <f>_xll.BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
-      <c r="AU57" s="1" t="n"/>
+        <f>BDP("MRSH US Equity","BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")</f>
+        <v/>
+      </c>
+      <c r="AT57" s="55" t="n"/>
+      <c r="AU57" s="60">
+        <f>BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","24Y")</f>
+        <v/>
+      </c>
       <c r="AV57" s="55">
-        <f>_xll.BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","24Y")</f>
+        <f>BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")</f>
         <v/>
       </c>
       <c r="AW57" s="55">
-        <f>_xll.BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")</f>
+        <f>BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")</f>
         <v/>
       </c>
       <c r="AX57" s="55">
-        <f>_xll.BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")</f>
+        <f>BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","27Y")</f>
         <v/>
       </c>
       <c r="AY57" s="55">
-        <f>_xll.BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AZ57" s="55">
-        <f>_xll.BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
-      <c r="BA57" s="1" t="n"/>
+        <f>BDP("MRSH US Equity","BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")</f>
+        <v/>
+      </c>
+      <c r="AZ57" s="55" t="n"/>
+      <c r="BA57" s="1">
+        <f>C57+BD57</f>
+        <v/>
+      </c>
       <c r="BB57" s="40">
-        <f>C57+BC57</f>
+        <f>AB57-AD57</f>
         <v/>
       </c>
       <c r="BC57" s="40">
-        <f>AC57-AE57</f>
-        <v/>
-      </c>
-      <c r="BD57" s="4">
         <f>C57</f>
         <v/>
       </c>
-      <c r="BE57" s="55">
-        <f>_xll.BDP("MRSH US Equity","TRAIL_12M_EBITDA")</f>
-        <v/>
-      </c>
+      <c r="BD57" s="55">
+        <f>BDP("MRSH US Equity","TRAIL_12M_EBITDA")</f>
+        <v/>
+      </c>
+      <c r="BE57" s="55" t="n"/>
       <c r="BF57" s="1" t="n"/>
       <c r="BG57" s="1" t="n"/>
       <c r="BH57" s="1" t="n"/>

</xml_diff>

<commit_message>
fix: clear BDP formulas from header, average, and category rows
</commit_message>
<xml_diff>
--- a/output/comp_sheet_updated.xlsx
+++ b/output/comp_sheet_updated.xlsx
@@ -12516,59 +12516,20 @@
         </is>
       </c>
       <c r="B65" s="1" t="n"/>
-      <c r="C65" s="43">
-        <f>BDP($B$65,"CUR_MKT_CAP")/1000000000</f>
-        <v/>
-      </c>
-      <c r="D65" s="44">
-        <f>BDP($B$65,"PX_LAST")</f>
-        <v/>
-      </c>
-      <c r="E65" s="45">
-        <f>IF(BDP($B$65,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")&lt;&gt;0,$D$65/BDP($B$65,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y"),"")</f>
-        <v/>
-      </c>
-      <c r="F65" s="45">
-        <f>IF(BDP($B$65,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&lt;&gt;0,$D$65/BDP($B$65,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y"),"")</f>
-        <v/>
-      </c>
-      <c r="G65" s="45">
-        <f>IF(BDP($B$65,"BEST_EPS","BEST_FPERIOD_OVERRIDE","29Y")&lt;&gt;0,$D$65/BDP($B$65,"BEST_EPS","BEST_FPERIOD_OVERRIDE","29Y"),"")</f>
-        <v/>
-      </c>
-      <c r="H65" s="43">
-        <f>BDP($B$65,"NET_DEBT_TO_EBITDA")</f>
-        <v/>
-      </c>
-      <c r="I65" s="43">
-        <f>BDP($B$65,"BEST_SALES","BEST_FPERIOD_OVERRIDE","27Y")/1000</f>
-        <v/>
-      </c>
-      <c r="J65" s="47">
-        <f>IF(BDP($B$65,"BEST_SALES","BEST_FPERIOD_OVERRIDE","27Y")&lt;&gt;0,BDP($B$65,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","27Y")/BDP($B$65,"BEST_SALES","BEST_FPERIOD_OVERRIDE","27Y"),"")</f>
-        <v/>
-      </c>
-      <c r="K65" s="43">
-        <f>BDP($B$65,"RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
-      <c r="L65" s="47">
-        <f>IF(AND(BDP($B$65,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")&gt;0,BDP($B$65,"BEST_SALES","BEST_FPERIOD_OVERRIDE","29Y")&gt;0),(BDP($B$65,"BEST_SALES","BEST_FPERIOD_OVERRIDE","29Y")/BDP($B$65,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="M65" s="47">
-        <f>IF(AND(BDP($B$65,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")&gt;0,BDP($B$65,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","29Y")&gt;0),(BDP($B$65,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","29Y")/BDP($B$65,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="N65" s="47">
-        <f>IF(AND(BDP($B$65,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")&gt;0,BDP($B$65,"BEST_EPS","BEST_FPERIOD_OVERRIDE","29Y")&gt;0),(BDP($B$65,"BEST_EPS","BEST_FPERIOD_OVERRIDE","29Y")/BDP($B$65,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
+      <c r="C65" s="43" t="n"/>
+      <c r="D65" s="44" t="n"/>
+      <c r="E65" s="45" t="n"/>
+      <c r="F65" s="45" t="n"/>
+      <c r="G65" s="45" t="n"/>
+      <c r="H65" s="43" t="n"/>
+      <c r="I65" s="43" t="n"/>
+      <c r="J65" s="47" t="n"/>
+      <c r="K65" s="43" t="n"/>
+      <c r="L65" s="47" t="n"/>
+      <c r="M65" s="47" t="n"/>
+      <c r="N65" s="47" t="n"/>
       <c r="O65" s="1" t="n"/>
-      <c r="P65" s="48">
-        <f>BDP($B$65,"CHG_PCT_YTD")/100</f>
-        <v/>
-      </c>
+      <c r="P65" s="48" t="n"/>
       <c r="Q65" s="1" t="n"/>
       <c r="R65" s="1" t="n"/>
       <c r="S65" s="42">
@@ -12586,97 +12547,34 @@
       <c r="X65" s="1" t="n"/>
       <c r="Y65" s="1" t="n"/>
       <c r="Z65" s="1" t="n"/>
-      <c r="AA65" s="48">
-        <f>BDP($B$65,"TRAIL_12M_OPER_INC")</f>
-        <v/>
-      </c>
-      <c r="AB65" s="43">
-        <f>BDP($B$65,"SHORT_AND_LONG_TERM_DEBT")</f>
-        <v/>
-      </c>
-      <c r="AC65" s="43">
-        <f>BDP($B$65,"TOTAL_EQUITY")</f>
-        <v/>
-      </c>
-      <c r="AD65" s="43">
-        <f>BDP($B$65,"BS_CASH_NEAR_CASH_ITEM")</f>
-        <v/>
-      </c>
-      <c r="AE65" s="43">
-        <f>BDP($B$65,"BS_LT_INVEST")</f>
-        <v/>
-      </c>
+      <c r="AA65" s="48" t="n"/>
+      <c r="AB65" s="43" t="n"/>
+      <c r="AC65" s="43" t="n"/>
+      <c r="AD65" s="43" t="n"/>
+      <c r="AE65" s="43" t="n"/>
       <c r="AF65" s="4">
         <f>AB65+AC65</f>
         <v/>
       </c>
-      <c r="AG65" s="43">
-        <f>BDP($B$65,"RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
+      <c r="AG65" s="43" t="n"/>
       <c r="AH65" s="41" t="n"/>
-      <c r="AI65" s="48">
-        <f>BDP($B$65,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AJ65" s="43">
-        <f>BDP($B$65,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AK65" s="43">
-        <f>BDP($B$65,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AL65" s="43">
-        <f>BDP($B$65,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
-      <c r="AM65" s="43">
-        <f>BDP($B$65,"BEST_EPS","BEST_FPERIOD_OVERRIDE","29Y")</f>
-        <v/>
-      </c>
+      <c r="AI65" s="48" t="n"/>
+      <c r="AJ65" s="43" t="n"/>
+      <c r="AK65" s="43" t="n"/>
+      <c r="AL65" s="43" t="n"/>
+      <c r="AM65" s="43" t="n"/>
       <c r="AN65" s="4" t="n"/>
-      <c r="AO65" s="48">
-        <f>BDP($B$65,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AP65" s="43">
-        <f>BDP($B$65,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AQ65" s="43">
-        <f>BDP($B$65,"BEST_SALES","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AR65" s="43">
-        <f>BDP($B$65,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
-      <c r="AS65" s="43">
-        <f>BDP($B$65,"BEST_SALES","BEST_FPERIOD_OVERRIDE","29Y")</f>
-        <v/>
-      </c>
+      <c r="AO65" s="48" t="n"/>
+      <c r="AP65" s="43" t="n"/>
+      <c r="AQ65" s="43" t="n"/>
+      <c r="AR65" s="43" t="n"/>
+      <c r="AS65" s="43" t="n"/>
       <c r="AT65" s="4" t="n"/>
-      <c r="AU65" s="48">
-        <f>BDP($B$65,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AV65" s="43">
-        <f>BDP($B$65,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AW65" s="43">
-        <f>BDP($B$65,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AX65" s="43">
-        <f>BDP($B$65,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
-      <c r="AY65" s="43">
-        <f>BDP($B$65,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","29Y")</f>
-        <v/>
-      </c>
+      <c r="AU65" s="48" t="n"/>
+      <c r="AV65" s="43" t="n"/>
+      <c r="AW65" s="43" t="n"/>
+      <c r="AX65" s="43" t="n"/>
+      <c r="AY65" s="43" t="n"/>
       <c r="AZ65" s="4" t="n"/>
       <c r="BA65" s="1">
         <f>C65+BD65</f>
@@ -12690,10 +12588,7 @@
         <f>C65</f>
         <v/>
       </c>
-      <c r="BD65" s="43">
-        <f>BDP($B$65,"TRAIL_12M_EBITDA")</f>
-        <v/>
-      </c>
+      <c r="BD65" s="43" t="n"/>
       <c r="BE65" s="4" t="n"/>
       <c r="BF65" s="1" t="n"/>
       <c r="BG65" s="1" t="n"/>
@@ -15287,59 +15182,20 @@
         </is>
       </c>
       <c r="B78" s="1" t="n"/>
-      <c r="C78" s="43">
-        <f>BDP($B$78,"CUR_MKT_CAP")/1000000000</f>
-        <v/>
-      </c>
-      <c r="D78" s="44">
-        <f>BDP($B$78,"PX_LAST")</f>
-        <v/>
-      </c>
-      <c r="E78" s="45">
-        <f>IF(BDP($B$78,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,$D$78/BDP($B$78,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
-        <v/>
-      </c>
-      <c r="F78" s="45">
-        <f>IF(BDP($B$78,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")&lt;&gt;0,$D$78/BDP($B$78,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y"),"")</f>
-        <v/>
-      </c>
-      <c r="G78" s="45">
-        <f>IF(BDP($B$78,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&lt;&gt;0,$D$78/BDP($B$78,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y"),"")</f>
-        <v/>
-      </c>
-      <c r="H78" s="43">
-        <f>BDP($B$78,"NET_DEBT_TO_EBITDA")</f>
-        <v/>
-      </c>
-      <c r="I78" s="43">
-        <f>BDP($B$78,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")/1000</f>
-        <v/>
-      </c>
-      <c r="J78" s="47">
-        <f>IF(BDP($B$78,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,BDP($B$78,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")/BDP($B$78,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
-        <v/>
-      </c>
-      <c r="K78" s="43">
-        <f>BDP($B$78,"RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
-      <c r="L78" s="47">
-        <f>IF(AND(BDP($B$78,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$78,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$78,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$78,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="M78" s="47">
-        <f>IF(AND(BDP($B$78,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$78,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$78,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$78,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="N78" s="47">
-        <f>IF(AND(BDP($B$78,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$78,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$78,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$78,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
+      <c r="C78" s="43" t="n"/>
+      <c r="D78" s="44" t="n"/>
+      <c r="E78" s="45" t="n"/>
+      <c r="F78" s="45" t="n"/>
+      <c r="G78" s="45" t="n"/>
+      <c r="H78" s="43" t="n"/>
+      <c r="I78" s="43" t="n"/>
+      <c r="J78" s="47" t="n"/>
+      <c r="K78" s="43" t="n"/>
+      <c r="L78" s="47" t="n"/>
+      <c r="M78" s="47" t="n"/>
+      <c r="N78" s="47" t="n"/>
       <c r="O78" s="1" t="n"/>
-      <c r="P78" s="48">
-        <f>BDP($B$78,"CHG_PCT_YTD")/100</f>
-        <v/>
-      </c>
+      <c r="P78" s="48" t="n"/>
       <c r="Q78" s="1" t="n"/>
       <c r="R78" s="1" t="n"/>
       <c r="S78" s="42">
@@ -15357,97 +15213,34 @@
       <c r="X78" s="1" t="n"/>
       <c r="Y78" s="1" t="n"/>
       <c r="Z78" s="1" t="n"/>
-      <c r="AA78" s="48">
-        <f>BDP($B$78,"TRAIL_12M_OPER_INC")</f>
-        <v/>
-      </c>
-      <c r="AB78" s="43">
-        <f>BDP($B$78,"SHORT_AND_LONG_TERM_DEBT")</f>
-        <v/>
-      </c>
-      <c r="AC78" s="43">
-        <f>BDP($B$78,"TOTAL_EQUITY")</f>
-        <v/>
-      </c>
-      <c r="AD78" s="43">
-        <f>BDP($B$78,"BS_CASH_NEAR_CASH_ITEM")</f>
-        <v/>
-      </c>
-      <c r="AE78" s="43">
-        <f>BDP($B$78,"BS_LT_INVEST")</f>
-        <v/>
-      </c>
+      <c r="AA78" s="48" t="n"/>
+      <c r="AB78" s="43" t="n"/>
+      <c r="AC78" s="43" t="n"/>
+      <c r="AD78" s="43" t="n"/>
+      <c r="AE78" s="43" t="n"/>
       <c r="AF78" s="4">
         <f>AB78+AC78</f>
         <v/>
       </c>
-      <c r="AG78" s="43">
-        <f>BDP($B$78,"RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
+      <c r="AG78" s="43" t="n"/>
       <c r="AH78" s="41" t="n"/>
-      <c r="AI78" s="48">
-        <f>BDP($B$78,"BEST_EPS","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AJ78" s="43">
-        <f>BDP($B$78,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AK78" s="43">
-        <f>BDP($B$78,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AL78" s="43">
-        <f>BDP($B$78,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AM78" s="43">
-        <f>BDP($B$78,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AI78" s="48" t="n"/>
+      <c r="AJ78" s="43" t="n"/>
+      <c r="AK78" s="43" t="n"/>
+      <c r="AL78" s="43" t="n"/>
+      <c r="AM78" s="43" t="n"/>
       <c r="AN78" s="4" t="n"/>
-      <c r="AO78" s="48">
-        <f>BDP($B$78,"BEST_SALES","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AP78" s="43">
-        <f>BDP($B$78,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AQ78" s="43">
-        <f>BDP($B$78,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AR78" s="43">
-        <f>BDP($B$78,"BEST_SALES","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AS78" s="43">
-        <f>BDP($B$78,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AO78" s="48" t="n"/>
+      <c r="AP78" s="43" t="n"/>
+      <c r="AQ78" s="43" t="n"/>
+      <c r="AR78" s="43" t="n"/>
+      <c r="AS78" s="43" t="n"/>
       <c r="AT78" s="4" t="n"/>
-      <c r="AU78" s="48">
-        <f>BDP($B$78,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AV78" s="43">
-        <f>BDP($B$78,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AW78" s="43">
-        <f>BDP($B$78,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AX78" s="43">
-        <f>BDP($B$78,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AY78" s="43">
-        <f>BDP($B$78,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AU78" s="48" t="n"/>
+      <c r="AV78" s="43" t="n"/>
+      <c r="AW78" s="43" t="n"/>
+      <c r="AX78" s="43" t="n"/>
+      <c r="AY78" s="43" t="n"/>
       <c r="AZ78" s="4" t="n"/>
       <c r="BA78" s="1">
         <f>C78+BD78</f>
@@ -15461,10 +15254,7 @@
         <f>C78</f>
         <v/>
       </c>
-      <c r="BD78" s="43">
-        <f>BDP($B$78,"TRAIL_12M_EBITDA")</f>
-        <v/>
-      </c>
+      <c r="BD78" s="43" t="n"/>
       <c r="BE78" s="4" t="n"/>
       <c r="BF78" s="1" t="n"/>
       <c r="BG78" s="1" t="n"/>
@@ -18334,59 +18124,20 @@
         </is>
       </c>
       <c r="B93" s="1" t="n"/>
-      <c r="C93" s="43">
-        <f>BDP($B$93,"CUR_MKT_CAP")/1000000000</f>
-        <v/>
-      </c>
-      <c r="D93" s="44">
-        <f>BDP($B$93,"PX_LAST")</f>
-        <v/>
-      </c>
-      <c r="E93" s="45">
-        <f>IF(BDP($B$93,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,$D$93/BDP($B$93,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
-        <v/>
-      </c>
-      <c r="F93" s="45">
-        <f>IF(BDP($B$93,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")&lt;&gt;0,$D$93/BDP($B$93,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y"),"")</f>
-        <v/>
-      </c>
-      <c r="G93" s="45">
-        <f>IF(BDP($B$93,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&lt;&gt;0,$D$93/BDP($B$93,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y"),"")</f>
-        <v/>
-      </c>
-      <c r="H93" s="46">
-        <f>BDP($B$93,"NET_DEBT_TO_EBITDA")</f>
-        <v/>
-      </c>
-      <c r="I93" s="43">
-        <f>BDP($B$93,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")/1000</f>
-        <v/>
-      </c>
-      <c r="J93" s="47">
-        <f>IF(BDP($B$93,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,BDP($B$93,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")/BDP($B$93,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
-        <v/>
-      </c>
-      <c r="K93" s="47">
-        <f>BDP($B$93,"RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
-      <c r="L93" s="47">
-        <f>IF(AND(BDP($B$93,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$93,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$93,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$93,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="M93" s="47">
-        <f>IF(AND(BDP($B$93,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$93,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$93,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$93,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="N93" s="47">
-        <f>IF(AND(BDP($B$93,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$93,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$93,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$93,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
+      <c r="C93" s="43" t="n"/>
+      <c r="D93" s="44" t="n"/>
+      <c r="E93" s="45" t="n"/>
+      <c r="F93" s="45" t="n"/>
+      <c r="G93" s="45" t="n"/>
+      <c r="H93" s="46" t="n"/>
+      <c r="I93" s="43" t="n"/>
+      <c r="J93" s="47" t="n"/>
+      <c r="K93" s="47" t="n"/>
+      <c r="L93" s="47" t="n"/>
+      <c r="M93" s="47" t="n"/>
+      <c r="N93" s="47" t="n"/>
       <c r="O93" s="1" t="n"/>
-      <c r="P93" s="47">
-        <f>BDP($B$93,"CHG_PCT_YTD")/100</f>
-        <v/>
-      </c>
+      <c r="P93" s="47" t="n"/>
       <c r="Q93" s="1" t="n"/>
       <c r="R93" s="1" t="n"/>
       <c r="S93" s="42">
@@ -18404,97 +18155,34 @@
       <c r="X93" s="1" t="n"/>
       <c r="Y93" s="1" t="n"/>
       <c r="Z93" s="1" t="n"/>
-      <c r="AA93" s="48">
-        <f>BDP($B$93,"TRAIL_12M_OPER_INC")</f>
-        <v/>
-      </c>
-      <c r="AB93" s="43">
-        <f>BDP($B$93,"SHORT_AND_LONG_TERM_DEBT")</f>
-        <v/>
-      </c>
-      <c r="AC93" s="43">
-        <f>BDP($B$93,"TOTAL_EQUITY")</f>
-        <v/>
-      </c>
-      <c r="AD93" s="43">
-        <f>BDP($B$93,"BS_CASH_NEAR_CASH_ITEM")</f>
-        <v/>
-      </c>
-      <c r="AE93" s="43">
-        <f>BDP($B$93,"BS_LT_INVEST")</f>
-        <v/>
-      </c>
+      <c r="AA93" s="48" t="n"/>
+      <c r="AB93" s="43" t="n"/>
+      <c r="AC93" s="43" t="n"/>
+      <c r="AD93" s="43" t="n"/>
+      <c r="AE93" s="43" t="n"/>
       <c r="AF93" s="4">
         <f>AB93+AC93</f>
         <v/>
       </c>
-      <c r="AG93" s="43">
-        <f>BDP($B$93,"RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
+      <c r="AG93" s="43" t="n"/>
       <c r="AH93" s="41" t="n"/>
-      <c r="AI93" s="48">
-        <f>BDP($B$93,"BEST_EPS","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AJ93" s="43">
-        <f>BDP($B$93,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AK93" s="43">
-        <f>BDP($B$93,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AL93" s="43">
-        <f>BDP($B$93,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AM93" s="43">
-        <f>BDP($B$93,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AI93" s="48" t="n"/>
+      <c r="AJ93" s="43" t="n"/>
+      <c r="AK93" s="43" t="n"/>
+      <c r="AL93" s="43" t="n"/>
+      <c r="AM93" s="43" t="n"/>
       <c r="AN93" s="4" t="n"/>
-      <c r="AO93" s="48">
-        <f>BDP($B$93,"BEST_SALES","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AP93" s="43">
-        <f>BDP($B$93,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AQ93" s="43">
-        <f>BDP($B$93,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AR93" s="43">
-        <f>BDP($B$93,"BEST_SALES","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AS93" s="43">
-        <f>BDP($B$93,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AO93" s="48" t="n"/>
+      <c r="AP93" s="43" t="n"/>
+      <c r="AQ93" s="43" t="n"/>
+      <c r="AR93" s="43" t="n"/>
+      <c r="AS93" s="43" t="n"/>
       <c r="AT93" s="4" t="n"/>
-      <c r="AU93" s="48">
-        <f>BDP($B$93,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AV93" s="43">
-        <f>BDP($B$93,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AW93" s="43">
-        <f>BDP($B$93,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AX93" s="43">
-        <f>BDP($B$93,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AY93" s="43">
-        <f>BDP($B$93,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AU93" s="48" t="n"/>
+      <c r="AV93" s="43" t="n"/>
+      <c r="AW93" s="43" t="n"/>
+      <c r="AX93" s="43" t="n"/>
+      <c r="AY93" s="43" t="n"/>
       <c r="AZ93" s="4" t="n"/>
       <c r="BA93" s="1">
         <f>C93+BD93</f>
@@ -18508,10 +18196,7 @@
         <f>C93</f>
         <v/>
       </c>
-      <c r="BD93" s="43">
-        <f>BDP($B$93,"TRAIL_12M_EBITDA")</f>
-        <v/>
-      </c>
+      <c r="BD93" s="43" t="n"/>
       <c r="BE93" s="4" t="n"/>
       <c r="BF93" s="1" t="n"/>
       <c r="BG93" s="1" t="n"/>
@@ -21893,59 +21578,20 @@
         </is>
       </c>
       <c r="B111" s="1" t="n"/>
-      <c r="C111" s="43">
-        <f>BDP($B$111,"CUR_MKT_CAP")/1000000000</f>
-        <v/>
-      </c>
-      <c r="D111" s="48">
-        <f>BDP($B$111,"PX_LAST")</f>
-        <v/>
-      </c>
-      <c r="E111" s="48">
-        <f>IF(BDP($B$111,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,$D$111/BDP($B$111,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
-        <v/>
-      </c>
-      <c r="F111" s="48">
-        <f>IF(BDP($B$111,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")&lt;&gt;0,$D$111/BDP($B$111,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y"),"")</f>
-        <v/>
-      </c>
-      <c r="G111" s="48">
-        <f>IF(BDP($B$111,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&lt;&gt;0,$D$111/BDP($B$111,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y"),"")</f>
-        <v/>
-      </c>
-      <c r="H111" s="48">
-        <f>BDP($B$111,"NET_DEBT_TO_EBITDA")</f>
-        <v/>
-      </c>
-      <c r="I111" s="48">
-        <f>BDP($B$111,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")/1000</f>
-        <v/>
-      </c>
-      <c r="J111" s="48">
-        <f>IF(BDP($B$111,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,BDP($B$111,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")/BDP($B$111,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
-        <v/>
-      </c>
-      <c r="K111" s="48">
-        <f>BDP($B$111,"RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
-      <c r="L111" s="48">
-        <f>IF(AND(BDP($B$111,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$111,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$111,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$111,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="M111" s="48">
-        <f>IF(AND(BDP($B$111,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$111,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$111,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$111,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="N111" s="48">
-        <f>IF(AND(BDP($B$111,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$111,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$111,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$111,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
+      <c r="C111" s="43" t="n"/>
+      <c r="D111" s="48" t="n"/>
+      <c r="E111" s="48" t="n"/>
+      <c r="F111" s="48" t="n"/>
+      <c r="G111" s="48" t="n"/>
+      <c r="H111" s="48" t="n"/>
+      <c r="I111" s="48" t="n"/>
+      <c r="J111" s="48" t="n"/>
+      <c r="K111" s="48" t="n"/>
+      <c r="L111" s="48" t="n"/>
+      <c r="M111" s="48" t="n"/>
+      <c r="N111" s="48" t="n"/>
       <c r="O111" s="1" t="n"/>
-      <c r="P111" s="48">
-        <f>BDP($B$111,"CHG_PCT_YTD")/100</f>
-        <v/>
-      </c>
+      <c r="P111" s="48" t="n"/>
       <c r="Q111" s="1" t="n"/>
       <c r="R111" s="1" t="n"/>
       <c r="S111" s="1">
@@ -21963,97 +21609,34 @@
       <c r="X111" s="1" t="n"/>
       <c r="Y111" s="1" t="n"/>
       <c r="Z111" s="1" t="n"/>
-      <c r="AA111" s="48">
-        <f>BDP($B$111,"TRAIL_12M_OPER_INC")</f>
-        <v/>
-      </c>
-      <c r="AB111" s="48">
-        <f>BDP($B$111,"SHORT_AND_LONG_TERM_DEBT")</f>
-        <v/>
-      </c>
-      <c r="AC111" s="48">
-        <f>BDP($B$111,"TOTAL_EQUITY")</f>
-        <v/>
-      </c>
-      <c r="AD111" s="48">
-        <f>BDP($B$111,"BS_CASH_NEAR_CASH_ITEM")</f>
-        <v/>
-      </c>
-      <c r="AE111" s="48">
-        <f>BDP($B$111,"BS_LT_INVEST")</f>
-        <v/>
-      </c>
+      <c r="AA111" s="48" t="n"/>
+      <c r="AB111" s="48" t="n"/>
+      <c r="AC111" s="48" t="n"/>
+      <c r="AD111" s="48" t="n"/>
+      <c r="AE111" s="48" t="n"/>
       <c r="AF111" s="1">
         <f>AB111+AC111</f>
         <v/>
       </c>
-      <c r="AG111" s="48">
-        <f>BDP($B$111,"RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
+      <c r="AG111" s="48" t="n"/>
       <c r="AH111" s="1" t="n"/>
-      <c r="AI111" s="48">
-        <f>BDP($B$111,"BEST_EPS","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AJ111" s="48">
-        <f>BDP($B$111,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AK111" s="48">
-        <f>BDP($B$111,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AL111" s="48">
-        <f>BDP($B$111,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AM111" s="48">
-        <f>BDP($B$111,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AI111" s="48" t="n"/>
+      <c r="AJ111" s="48" t="n"/>
+      <c r="AK111" s="48" t="n"/>
+      <c r="AL111" s="48" t="n"/>
+      <c r="AM111" s="48" t="n"/>
       <c r="AN111" s="1" t="n"/>
-      <c r="AO111" s="48">
-        <f>BDP($B$111,"BEST_SALES","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AP111" s="48">
-        <f>BDP($B$111,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AQ111" s="48">
-        <f>BDP($B$111,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AR111" s="48">
-        <f>BDP($B$111,"BEST_SALES","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AS111" s="48">
-        <f>BDP($B$111,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AO111" s="48" t="n"/>
+      <c r="AP111" s="48" t="n"/>
+      <c r="AQ111" s="48" t="n"/>
+      <c r="AR111" s="48" t="n"/>
+      <c r="AS111" s="48" t="n"/>
       <c r="AT111" s="1" t="n"/>
-      <c r="AU111" s="48">
-        <f>BDP($B$111,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AV111" s="48">
-        <f>BDP($B$111,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AW111" s="48">
-        <f>BDP($B$111,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AX111" s="48">
-        <f>BDP($B$111,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AY111" s="48">
-        <f>BDP($B$111,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AU111" s="48" t="n"/>
+      <c r="AV111" s="48" t="n"/>
+      <c r="AW111" s="48" t="n"/>
+      <c r="AX111" s="48" t="n"/>
+      <c r="AY111" s="48" t="n"/>
       <c r="AZ111" s="1" t="n"/>
       <c r="BA111" s="1">
         <f>C111+BD111</f>
@@ -22067,10 +21650,7 @@
         <f>C111</f>
         <v/>
       </c>
-      <c r="BD111" s="48">
-        <f>BDP($B$111,"TRAIL_12M_EBITDA")</f>
-        <v/>
-      </c>
+      <c r="BD111" s="48" t="n"/>
       <c r="BE111" s="1" t="n"/>
       <c r="BF111" s="1" t="n"/>
       <c r="BG111" s="1" t="n"/>
@@ -25437,59 +25017,20 @@
         </is>
       </c>
       <c r="B130" s="1" t="n"/>
-      <c r="C130" s="48">
-        <f>BDP($B$130,"CUR_MKT_CAP")/1000000000</f>
-        <v/>
-      </c>
-      <c r="D130" s="48">
-        <f>BDP($B$130,"PX_LAST")</f>
-        <v/>
-      </c>
-      <c r="E130" s="48">
-        <f>IF(BDP($B$130,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,$D$130/BDP($B$130,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
-        <v/>
-      </c>
-      <c r="F130" s="48">
-        <f>IF(BDP($B$130,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")&lt;&gt;0,$D$130/BDP($B$130,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y"),"")</f>
-        <v/>
-      </c>
-      <c r="G130" s="48">
-        <f>IF(BDP($B$130,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&lt;&gt;0,$D$130/BDP($B$130,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y"),"")</f>
-        <v/>
-      </c>
-      <c r="H130" s="48">
-        <f>BDP($B$130,"NET_DEBT_TO_EBITDA")</f>
-        <v/>
-      </c>
-      <c r="I130" s="48">
-        <f>BDP($B$130,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")/1000</f>
-        <v/>
-      </c>
-      <c r="J130" s="48">
-        <f>IF(BDP($B$130,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,BDP($B$130,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")/BDP($B$130,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
-        <v/>
-      </c>
-      <c r="K130" s="48">
-        <f>BDP($B$130,"RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
-      <c r="L130" s="48">
-        <f>IF(AND(BDP($B$130,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$130,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$130,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$130,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="M130" s="48">
-        <f>IF(AND(BDP($B$130,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$130,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$130,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$130,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="N130" s="48">
-        <f>IF(AND(BDP($B$130,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$130,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$130,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$130,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
+      <c r="C130" s="48" t="n"/>
+      <c r="D130" s="48" t="n"/>
+      <c r="E130" s="48" t="n"/>
+      <c r="F130" s="48" t="n"/>
+      <c r="G130" s="48" t="n"/>
+      <c r="H130" s="48" t="n"/>
+      <c r="I130" s="48" t="n"/>
+      <c r="J130" s="48" t="n"/>
+      <c r="K130" s="48" t="n"/>
+      <c r="L130" s="48" t="n"/>
+      <c r="M130" s="48" t="n"/>
+      <c r="N130" s="48" t="n"/>
       <c r="O130" s="1" t="n"/>
-      <c r="P130" s="48">
-        <f>BDP($B$130,"CHG_PCT_YTD")/100</f>
-        <v/>
-      </c>
+      <c r="P130" s="48" t="n"/>
       <c r="Q130" s="1" t="n"/>
       <c r="R130" s="1" t="n"/>
       <c r="S130" s="1">
@@ -25507,97 +25048,34 @@
       <c r="X130" s="1" t="n"/>
       <c r="Y130" s="1" t="n"/>
       <c r="Z130" s="1" t="n"/>
-      <c r="AA130" s="48">
-        <f>BDP($B$130,"TRAIL_12M_OPER_INC")</f>
-        <v/>
-      </c>
-      <c r="AB130" s="48">
-        <f>BDP($B$130,"SHORT_AND_LONG_TERM_DEBT")</f>
-        <v/>
-      </c>
-      <c r="AC130" s="48">
-        <f>BDP($B$130,"TOTAL_EQUITY")</f>
-        <v/>
-      </c>
-      <c r="AD130" s="48">
-        <f>BDP($B$130,"BS_CASH_NEAR_CASH_ITEM")</f>
-        <v/>
-      </c>
-      <c r="AE130" s="48">
-        <f>BDP($B$130,"BS_LT_INVEST")</f>
-        <v/>
-      </c>
+      <c r="AA130" s="48" t="n"/>
+      <c r="AB130" s="48" t="n"/>
+      <c r="AC130" s="48" t="n"/>
+      <c r="AD130" s="48" t="n"/>
+      <c r="AE130" s="48" t="n"/>
       <c r="AF130" s="1">
         <f>AB130+AC130</f>
         <v/>
       </c>
-      <c r="AG130" s="48">
-        <f>BDP($B$130,"RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
+      <c r="AG130" s="48" t="n"/>
       <c r="AH130" s="1" t="n"/>
-      <c r="AI130" s="48">
-        <f>BDP($B$130,"BEST_EPS","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AJ130" s="48">
-        <f>BDP($B$130,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AK130" s="48">
-        <f>BDP($B$130,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AL130" s="48">
-        <f>BDP($B$130,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AM130" s="48">
-        <f>BDP($B$130,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AI130" s="48" t="n"/>
+      <c r="AJ130" s="48" t="n"/>
+      <c r="AK130" s="48" t="n"/>
+      <c r="AL130" s="48" t="n"/>
+      <c r="AM130" s="48" t="n"/>
       <c r="AN130" s="1" t="n"/>
-      <c r="AO130" s="48">
-        <f>BDP($B$130,"BEST_SALES","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AP130" s="48">
-        <f>BDP($B$130,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AQ130" s="48">
-        <f>BDP($B$130,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AR130" s="48">
-        <f>BDP($B$130,"BEST_SALES","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AS130" s="48">
-        <f>BDP($B$130,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AO130" s="48" t="n"/>
+      <c r="AP130" s="48" t="n"/>
+      <c r="AQ130" s="48" t="n"/>
+      <c r="AR130" s="48" t="n"/>
+      <c r="AS130" s="48" t="n"/>
       <c r="AT130" s="1" t="n"/>
-      <c r="AU130" s="48">
-        <f>BDP($B$130,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AV130" s="48">
-        <f>BDP($B$130,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AW130" s="48">
-        <f>BDP($B$130,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AX130" s="48">
-        <f>BDP($B$130,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AY130" s="48">
-        <f>BDP($B$130,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AU130" s="48" t="n"/>
+      <c r="AV130" s="48" t="n"/>
+      <c r="AW130" s="48" t="n"/>
+      <c r="AX130" s="48" t="n"/>
+      <c r="AY130" s="48" t="n"/>
       <c r="AZ130" s="1" t="n"/>
       <c r="BA130" s="1">
         <f>C130+BD130</f>
@@ -25611,10 +25089,7 @@
         <f>C130</f>
         <v/>
       </c>
-      <c r="BD130" s="48">
-        <f>BDP($B$130,"TRAIL_12M_EBITDA")</f>
-        <v/>
-      </c>
+      <c r="BD130" s="48" t="n"/>
       <c r="BE130" s="1" t="n"/>
       <c r="BF130" s="1" t="n"/>
       <c r="BG130" s="1" t="n"/>
@@ -26849,59 +26324,20 @@
         </is>
       </c>
       <c r="B137" s="1" t="n"/>
-      <c r="C137" s="48">
-        <f>BDP($B$137,"CUR_MKT_CAP")/1000000000</f>
-        <v/>
-      </c>
-      <c r="D137" s="48">
-        <f>BDP($B$137,"PX_LAST")</f>
-        <v/>
-      </c>
-      <c r="E137" s="48">
-        <f>IF(BDP($B$137,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,$D$137/BDP($B$137,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
-        <v/>
-      </c>
-      <c r="F137" s="48">
-        <f>IF(BDP($B$137,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")&lt;&gt;0,$D$137/BDP($B$137,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y"),"")</f>
-        <v/>
-      </c>
-      <c r="G137" s="48">
-        <f>IF(BDP($B$137,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&lt;&gt;0,$D$137/BDP($B$137,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y"),"")</f>
-        <v/>
-      </c>
-      <c r="H137" s="48">
-        <f>BDP($B$137,"NET_DEBT_TO_EBITDA")</f>
-        <v/>
-      </c>
-      <c r="I137" s="48">
-        <f>BDP($B$137,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")/1000</f>
-        <v/>
-      </c>
-      <c r="J137" s="48">
-        <f>IF(BDP($B$137,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,BDP($B$137,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")/BDP($B$137,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
-        <v/>
-      </c>
-      <c r="K137" s="48">
-        <f>BDP($B$137,"RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
-      <c r="L137" s="48">
-        <f>IF(AND(BDP($B$137,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$137,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$137,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$137,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="M137" s="48">
-        <f>IF(AND(BDP($B$137,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$137,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$137,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$137,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="N137" s="48">
-        <f>IF(AND(BDP($B$137,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$137,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$137,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$137,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
+      <c r="C137" s="48" t="n"/>
+      <c r="D137" s="48" t="n"/>
+      <c r="E137" s="48" t="n"/>
+      <c r="F137" s="48" t="n"/>
+      <c r="G137" s="48" t="n"/>
+      <c r="H137" s="48" t="n"/>
+      <c r="I137" s="48" t="n"/>
+      <c r="J137" s="48" t="n"/>
+      <c r="K137" s="48" t="n"/>
+      <c r="L137" s="48" t="n"/>
+      <c r="M137" s="48" t="n"/>
+      <c r="N137" s="48" t="n"/>
       <c r="O137" s="1" t="n"/>
-      <c r="P137" s="48">
-        <f>BDP($B$137,"CHG_PCT_YTD")/100</f>
-        <v/>
-      </c>
+      <c r="P137" s="48" t="n"/>
       <c r="Q137" s="1" t="n"/>
       <c r="R137" s="1" t="n"/>
       <c r="S137" s="1">
@@ -26919,97 +26355,34 @@
       <c r="X137" s="1" t="n"/>
       <c r="Y137" s="1" t="n"/>
       <c r="Z137" s="1" t="n"/>
-      <c r="AA137" s="47">
-        <f>BDP($B$137,"TRAIL_12M_OPER_INC")</f>
-        <v/>
-      </c>
-      <c r="AB137" s="48">
-        <f>BDP($B$137,"SHORT_AND_LONG_TERM_DEBT")</f>
-        <v/>
-      </c>
-      <c r="AC137" s="48">
-        <f>BDP($B$137,"TOTAL_EQUITY")</f>
-        <v/>
-      </c>
-      <c r="AD137" s="48">
-        <f>BDP($B$137,"BS_CASH_NEAR_CASH_ITEM")</f>
-        <v/>
-      </c>
-      <c r="AE137" s="48">
-        <f>BDP($B$137,"BS_LT_INVEST")</f>
-        <v/>
-      </c>
+      <c r="AA137" s="47" t="n"/>
+      <c r="AB137" s="48" t="n"/>
+      <c r="AC137" s="48" t="n"/>
+      <c r="AD137" s="48" t="n"/>
+      <c r="AE137" s="48" t="n"/>
       <c r="AF137" s="1">
         <f>AB137+AC137</f>
         <v/>
       </c>
-      <c r="AG137" s="48">
-        <f>BDP($B$137,"RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
+      <c r="AG137" s="48" t="n"/>
       <c r="AH137" s="1" t="n"/>
-      <c r="AI137" s="48">
-        <f>BDP($B$137,"BEST_EPS","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AJ137" s="48">
-        <f>BDP($B$137,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AK137" s="48">
-        <f>BDP($B$137,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AL137" s="48">
-        <f>BDP($B$137,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AM137" s="48">
-        <f>BDP($B$137,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AI137" s="48" t="n"/>
+      <c r="AJ137" s="48" t="n"/>
+      <c r="AK137" s="48" t="n"/>
+      <c r="AL137" s="48" t="n"/>
+      <c r="AM137" s="48" t="n"/>
       <c r="AN137" s="1" t="n"/>
-      <c r="AO137" s="48">
-        <f>BDP($B$137,"BEST_SALES","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AP137" s="48">
-        <f>BDP($B$137,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AQ137" s="48">
-        <f>BDP($B$137,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AR137" s="48">
-        <f>BDP($B$137,"BEST_SALES","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AS137" s="48">
-        <f>BDP($B$137,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AO137" s="48" t="n"/>
+      <c r="AP137" s="48" t="n"/>
+      <c r="AQ137" s="48" t="n"/>
+      <c r="AR137" s="48" t="n"/>
+      <c r="AS137" s="48" t="n"/>
       <c r="AT137" s="1" t="n"/>
-      <c r="AU137" s="48">
-        <f>BDP($B$137,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AV137" s="48">
-        <f>BDP($B$137,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AW137" s="48">
-        <f>BDP($B$137,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AX137" s="48">
-        <f>BDP($B$137,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AY137" s="48">
-        <f>BDP($B$137,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AU137" s="48" t="n"/>
+      <c r="AV137" s="48" t="n"/>
+      <c r="AW137" s="48" t="n"/>
+      <c r="AX137" s="48" t="n"/>
+      <c r="AY137" s="48" t="n"/>
       <c r="AZ137" s="1" t="n"/>
       <c r="BA137" s="1">
         <f>C137+BD137</f>
@@ -27023,10 +26396,7 @@
         <f>C137</f>
         <v/>
       </c>
-      <c r="BD137" s="48">
-        <f>BDP($B$137,"TRAIL_12M_EBITDA")</f>
-        <v/>
-      </c>
+      <c r="BD137" s="48" t="n"/>
       <c r="BE137" s="1" t="n"/>
       <c r="BF137" s="1" t="n"/>
       <c r="BG137" s="1" t="n"/>
@@ -27817,59 +27187,20 @@
         </is>
       </c>
       <c r="B142" s="1" t="n"/>
-      <c r="C142" s="43">
-        <f>BDP($B$142,"CUR_MKT_CAP")/1000000000</f>
-        <v/>
-      </c>
-      <c r="D142" s="44">
-        <f>BDP($B$142,"PX_LAST")</f>
-        <v/>
-      </c>
-      <c r="E142" s="45">
-        <f>IF(BDP($B$142,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,$D$142/BDP($B$142,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
-        <v/>
-      </c>
-      <c r="F142" s="45">
-        <f>IF(BDP($B$142,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")&lt;&gt;0,$D$142/BDP($B$142,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y"),"")</f>
-        <v/>
-      </c>
-      <c r="G142" s="45">
-        <f>IF(BDP($B$142,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&lt;&gt;0,$D$142/BDP($B$142,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y"),"")</f>
-        <v/>
-      </c>
-      <c r="H142" s="46">
-        <f>BDP($B$142,"NET_DEBT_TO_EBITDA")</f>
-        <v/>
-      </c>
-      <c r="I142" s="43">
-        <f>BDP($B$142,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")/1000</f>
-        <v/>
-      </c>
-      <c r="J142" s="47">
-        <f>IF(BDP($B$142,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,BDP($B$142,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")/BDP($B$142,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
-        <v/>
-      </c>
-      <c r="K142" s="47">
-        <f>BDP($B$142,"RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
-      <c r="L142" s="47">
-        <f>IF(AND(BDP($B$142,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$142,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$142,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$142,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="M142" s="47">
-        <f>IF(AND(BDP($B$142,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$142,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$142,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$142,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="N142" s="47">
-        <f>IF(AND(BDP($B$142,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$142,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$142,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$142,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
+      <c r="C142" s="43" t="n"/>
+      <c r="D142" s="44" t="n"/>
+      <c r="E142" s="45" t="n"/>
+      <c r="F142" s="45" t="n"/>
+      <c r="G142" s="45" t="n"/>
+      <c r="H142" s="46" t="n"/>
+      <c r="I142" s="43" t="n"/>
+      <c r="J142" s="47" t="n"/>
+      <c r="K142" s="47" t="n"/>
+      <c r="L142" s="47" t="n"/>
+      <c r="M142" s="47" t="n"/>
+      <c r="N142" s="47" t="n"/>
       <c r="O142" s="1" t="n"/>
-      <c r="P142" s="48">
-        <f>BDP($B$142,"CHG_PCT_YTD")/100</f>
-        <v/>
-      </c>
+      <c r="P142" s="48" t="n"/>
       <c r="Q142" s="1" t="n"/>
       <c r="R142" s="1" t="n"/>
       <c r="S142" s="42">
@@ -27887,97 +27218,34 @@
       <c r="X142" s="1" t="n"/>
       <c r="Y142" s="1" t="n"/>
       <c r="Z142" s="1" t="n"/>
-      <c r="AA142" s="47">
-        <f>BDP($B$142,"TRAIL_12M_OPER_INC")</f>
-        <v/>
-      </c>
-      <c r="AB142" s="43">
-        <f>BDP($B$142,"SHORT_AND_LONG_TERM_DEBT")</f>
-        <v/>
-      </c>
-      <c r="AC142" s="43">
-        <f>BDP($B$142,"TOTAL_EQUITY")</f>
-        <v/>
-      </c>
-      <c r="AD142" s="43">
-        <f>BDP($B$142,"BS_CASH_NEAR_CASH_ITEM")</f>
-        <v/>
-      </c>
-      <c r="AE142" s="43">
-        <f>BDP($B$142,"BS_LT_INVEST")</f>
-        <v/>
-      </c>
+      <c r="AA142" s="47" t="n"/>
+      <c r="AB142" s="43" t="n"/>
+      <c r="AC142" s="43" t="n"/>
+      <c r="AD142" s="43" t="n"/>
+      <c r="AE142" s="43" t="n"/>
       <c r="AF142" s="4">
         <f>AB142+AC142</f>
         <v/>
       </c>
-      <c r="AG142" s="43">
-        <f>BDP($B$142,"RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
+      <c r="AG142" s="43" t="n"/>
       <c r="AH142" s="41" t="n"/>
-      <c r="AI142" s="48">
-        <f>BDP($B$142,"BEST_EPS","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AJ142" s="43">
-        <f>BDP($B$142,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AK142" s="43">
-        <f>BDP($B$142,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AL142" s="43">
-        <f>BDP($B$142,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AM142" s="43">
-        <f>BDP($B$142,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AI142" s="48" t="n"/>
+      <c r="AJ142" s="43" t="n"/>
+      <c r="AK142" s="43" t="n"/>
+      <c r="AL142" s="43" t="n"/>
+      <c r="AM142" s="43" t="n"/>
       <c r="AN142" s="4" t="n"/>
-      <c r="AO142" s="43">
-        <f>BDP($B$142,"BEST_SALES","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AP142" s="43">
-        <f>BDP($B$142,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AQ142" s="43">
-        <f>BDP($B$142,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AR142" s="43">
-        <f>BDP($B$142,"BEST_SALES","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AS142" s="43">
-        <f>BDP($B$142,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AO142" s="43" t="n"/>
+      <c r="AP142" s="43" t="n"/>
+      <c r="AQ142" s="43" t="n"/>
+      <c r="AR142" s="43" t="n"/>
+      <c r="AS142" s="43" t="n"/>
       <c r="AT142" s="4" t="n"/>
-      <c r="AU142" s="48">
-        <f>BDP($B$142,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AV142" s="43">
-        <f>BDP($B$142,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AW142" s="43">
-        <f>BDP($B$142,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AX142" s="43">
-        <f>BDP($B$142,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AY142" s="43">
-        <f>BDP($B$142,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AU142" s="48" t="n"/>
+      <c r="AV142" s="43" t="n"/>
+      <c r="AW142" s="43" t="n"/>
+      <c r="AX142" s="43" t="n"/>
+      <c r="AY142" s="43" t="n"/>
       <c r="AZ142" s="4" t="n"/>
       <c r="BA142" s="1">
         <f>C142+BD142</f>
@@ -27991,10 +27259,7 @@
         <f>C142</f>
         <v/>
       </c>
-      <c r="BD142" s="43">
-        <f>BDP($B$142,"TRAIL_12M_EBITDA")</f>
-        <v/>
-      </c>
+      <c r="BD142" s="43" t="n"/>
       <c r="BE142" s="4" t="n"/>
       <c r="BF142" s="1" t="n"/>
       <c r="BG142" s="1" t="n"/>
@@ -28719,59 +27984,20 @@
         </is>
       </c>
       <c r="B147" s="1" t="n"/>
-      <c r="C147" s="43">
-        <f>BDP($B$147,"CUR_MKT_CAP")/1000000000</f>
-        <v/>
-      </c>
-      <c r="D147" s="44">
-        <f>BDP($B$147,"PX_LAST")</f>
-        <v/>
-      </c>
-      <c r="E147" s="45">
-        <f>IF(BDP($B$147,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,$D$147/BDP($B$147,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
-        <v/>
-      </c>
-      <c r="F147" s="45">
-        <f>IF(BDP($B$147,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")&lt;&gt;0,$D$147/BDP($B$147,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y"),"")</f>
-        <v/>
-      </c>
-      <c r="G147" s="45">
-        <f>IF(BDP($B$147,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&lt;&gt;0,$D$147/BDP($B$147,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y"),"")</f>
-        <v/>
-      </c>
-      <c r="H147" s="46">
-        <f>BDP($B$147,"NET_DEBT_TO_EBITDA")</f>
-        <v/>
-      </c>
-      <c r="I147" s="43">
-        <f>BDP($B$147,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")/1000</f>
-        <v/>
-      </c>
-      <c r="J147" s="47">
-        <f>IF(BDP($B$147,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,BDP($B$147,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")/BDP($B$147,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
-        <v/>
-      </c>
-      <c r="K147" s="47">
-        <f>BDP($B$147,"RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
-      <c r="L147" s="47">
-        <f>IF(AND(BDP($B$147,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$147,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$147,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$147,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="M147" s="47">
-        <f>IF(AND(BDP($B$147,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$147,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$147,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$147,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="N147" s="47">
-        <f>IF(AND(BDP($B$147,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$147,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$147,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$147,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
+      <c r="C147" s="43" t="n"/>
+      <c r="D147" s="44" t="n"/>
+      <c r="E147" s="45" t="n"/>
+      <c r="F147" s="45" t="n"/>
+      <c r="G147" s="45" t="n"/>
+      <c r="H147" s="46" t="n"/>
+      <c r="I147" s="43" t="n"/>
+      <c r="J147" s="47" t="n"/>
+      <c r="K147" s="47" t="n"/>
+      <c r="L147" s="47" t="n"/>
+      <c r="M147" s="47" t="n"/>
+      <c r="N147" s="47" t="n"/>
       <c r="O147" s="1" t="n"/>
-      <c r="P147" s="48">
-        <f>BDP($B$147,"CHG_PCT_YTD")/100</f>
-        <v/>
-      </c>
+      <c r="P147" s="48" t="n"/>
       <c r="Q147" s="1" t="n"/>
       <c r="R147" s="1" t="n"/>
       <c r="S147" s="42">
@@ -28789,97 +28015,34 @@
       <c r="X147" s="1" t="n"/>
       <c r="Y147" s="1" t="n"/>
       <c r="Z147" s="1" t="n"/>
-      <c r="AA147" s="47">
-        <f>BDP($B$147,"TRAIL_12M_OPER_INC")</f>
-        <v/>
-      </c>
-      <c r="AB147" s="43">
-        <f>BDP($B$147,"SHORT_AND_LONG_TERM_DEBT")</f>
-        <v/>
-      </c>
-      <c r="AC147" s="43">
-        <f>BDP($B$147,"TOTAL_EQUITY")</f>
-        <v/>
-      </c>
-      <c r="AD147" s="43">
-        <f>BDP($B$147,"BS_CASH_NEAR_CASH_ITEM")</f>
-        <v/>
-      </c>
-      <c r="AE147" s="43">
-        <f>BDP($B$147,"BS_LT_INVEST")</f>
-        <v/>
-      </c>
+      <c r="AA147" s="47" t="n"/>
+      <c r="AB147" s="43" t="n"/>
+      <c r="AC147" s="43" t="n"/>
+      <c r="AD147" s="43" t="n"/>
+      <c r="AE147" s="43" t="n"/>
       <c r="AF147" s="4">
         <f>AB147+AC147</f>
         <v/>
       </c>
-      <c r="AG147" s="43">
-        <f>BDP($B$147,"RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
+      <c r="AG147" s="43" t="n"/>
       <c r="AH147" s="41" t="n"/>
-      <c r="AI147" s="48">
-        <f>BDP($B$147,"BEST_EPS","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AJ147" s="43">
-        <f>BDP($B$147,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AK147" s="43">
-        <f>BDP($B$147,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AL147" s="43">
-        <f>BDP($B$147,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AM147" s="43">
-        <f>BDP($B$147,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AI147" s="48" t="n"/>
+      <c r="AJ147" s="43" t="n"/>
+      <c r="AK147" s="43" t="n"/>
+      <c r="AL147" s="43" t="n"/>
+      <c r="AM147" s="43" t="n"/>
       <c r="AN147" s="4" t="n"/>
-      <c r="AO147" s="43">
-        <f>BDP($B$147,"BEST_SALES","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AP147" s="43">
-        <f>BDP($B$147,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AQ147" s="43">
-        <f>BDP($B$147,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AR147" s="43">
-        <f>BDP($B$147,"BEST_SALES","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AS147" s="43">
-        <f>BDP($B$147,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AO147" s="43" t="n"/>
+      <c r="AP147" s="43" t="n"/>
+      <c r="AQ147" s="43" t="n"/>
+      <c r="AR147" s="43" t="n"/>
+      <c r="AS147" s="43" t="n"/>
       <c r="AT147" s="4" t="n"/>
-      <c r="AU147" s="48">
-        <f>BDP($B$147,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AV147" s="43">
-        <f>BDP($B$147,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AW147" s="43">
-        <f>BDP($B$147,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AX147" s="43">
-        <f>BDP($B$147,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AY147" s="43">
-        <f>BDP($B$147,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AU147" s="48" t="n"/>
+      <c r="AV147" s="43" t="n"/>
+      <c r="AW147" s="43" t="n"/>
+      <c r="AX147" s="43" t="n"/>
+      <c r="AY147" s="43" t="n"/>
       <c r="AZ147" s="4" t="n"/>
       <c r="BA147" s="1">
         <f>C147+BD147</f>
@@ -28893,10 +28056,7 @@
         <f>C147</f>
         <v/>
       </c>
-      <c r="BD147" s="43">
-        <f>BDP($B$147,"TRAIL_12M_EBITDA")</f>
-        <v/>
-      </c>
+      <c r="BD147" s="43" t="n"/>
       <c r="BE147" s="4" t="n"/>
       <c r="BF147" s="1" t="n"/>
       <c r="BG147" s="1" t="n"/>
@@ -31907,59 +31067,20 @@
         </is>
       </c>
       <c r="B162" s="1" t="n"/>
-      <c r="C162" s="43">
-        <f>BDP($B$162,"CUR_MKT_CAP")/1000000000</f>
-        <v/>
-      </c>
-      <c r="D162" s="44">
-        <f>BDP($B$162,"PX_LAST")</f>
-        <v/>
-      </c>
-      <c r="E162" s="45">
-        <f>IF(BDP($B$162,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,$D$162/BDP($B$162,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
-        <v/>
-      </c>
-      <c r="F162" s="45">
-        <f>IF(BDP($B$162,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")&lt;&gt;0,$D$162/BDP($B$162,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y"),"")</f>
-        <v/>
-      </c>
-      <c r="G162" s="45">
-        <f>IF(BDP($B$162,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&lt;&gt;0,$D$162/BDP($B$162,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y"),"")</f>
-        <v/>
-      </c>
-      <c r="H162" s="46">
-        <f>BDP($B$162,"NET_DEBT_TO_EBITDA")</f>
-        <v/>
-      </c>
-      <c r="I162" s="43">
-        <f>BDP($B$162,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")/1000</f>
-        <v/>
-      </c>
-      <c r="J162" s="47">
-        <f>IF(BDP($B$162,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")&lt;&gt;0,BDP($B$162,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")/BDP($B$162,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y"),"")</f>
-        <v/>
-      </c>
-      <c r="K162" s="47">
-        <f>BDP($B$162,"RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
-      <c r="L162" s="47">
-        <f>IF(AND(BDP($B$162,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$162,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$162,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$162,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="M162" s="47">
-        <f>IF(AND(BDP($B$162,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$162,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$162,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$162,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
-      <c r="N162" s="47">
-        <f>IF(AND(BDP($B$162,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")&gt;0,BDP($B$162,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")&gt;0),(BDP($B$162,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")/BDP($B$162,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y"))^(1/3)-1,"")</f>
-        <v/>
-      </c>
+      <c r="C162" s="43" t="n"/>
+      <c r="D162" s="44" t="n"/>
+      <c r="E162" s="45" t="n"/>
+      <c r="F162" s="45" t="n"/>
+      <c r="G162" s="45" t="n"/>
+      <c r="H162" s="46" t="n"/>
+      <c r="I162" s="43" t="n"/>
+      <c r="J162" s="47" t="n"/>
+      <c r="K162" s="47" t="n"/>
+      <c r="L162" s="47" t="n"/>
+      <c r="M162" s="47" t="n"/>
+      <c r="N162" s="47" t="n"/>
       <c r="O162" s="1" t="n"/>
-      <c r="P162" s="48">
-        <f>BDP($B$162,"CHG_PCT_YTD")/100</f>
-        <v/>
-      </c>
+      <c r="P162" s="48" t="n"/>
       <c r="Q162" s="1" t="n"/>
       <c r="R162" s="1" t="n"/>
       <c r="S162" s="40">
@@ -31977,97 +31098,34 @@
       <c r="X162" s="1" t="n"/>
       <c r="Y162" s="1" t="n"/>
       <c r="Z162" s="1" t="n"/>
-      <c r="AA162" s="48">
-        <f>BDP($B$162,"TRAIL_12M_OPER_INC")</f>
-        <v/>
-      </c>
-      <c r="AB162" s="43">
-        <f>BDP($B$162,"SHORT_AND_LONG_TERM_DEBT")</f>
-        <v/>
-      </c>
-      <c r="AC162" s="43">
-        <f>BDP($B$162,"TOTAL_EQUITY")</f>
-        <v/>
-      </c>
-      <c r="AD162" s="43">
-        <f>BDP($B$162,"BS_CASH_NEAR_CASH_ITEM")</f>
-        <v/>
-      </c>
-      <c r="AE162" s="43">
-        <f>BDP($B$162,"BS_LT_INVEST")</f>
-        <v/>
-      </c>
+      <c r="AA162" s="48" t="n"/>
+      <c r="AB162" s="43" t="n"/>
+      <c r="AC162" s="43" t="n"/>
+      <c r="AD162" s="43" t="n"/>
+      <c r="AE162" s="43" t="n"/>
       <c r="AF162" s="4">
         <f>AB162+AC162</f>
         <v/>
       </c>
-      <c r="AG162" s="43">
-        <f>BDP($B$162,"RETURN_ON_INV_CAPITAL")/100</f>
-        <v/>
-      </c>
+      <c r="AG162" s="43" t="n"/>
       <c r="AH162" s="41" t="n"/>
-      <c r="AI162" s="48">
-        <f>BDP($B$162,"BEST_EPS","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AJ162" s="43">
-        <f>BDP($B$162,"BEST_EPS","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AK162" s="43">
-        <f>BDP($B$162,"BEST_EPS","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AL162" s="43">
-        <f>BDP($B$162,"BEST_EPS","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AM162" s="43">
-        <f>BDP($B$162,"BEST_EPS","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AI162" s="48" t="n"/>
+      <c r="AJ162" s="43" t="n"/>
+      <c r="AK162" s="43" t="n"/>
+      <c r="AL162" s="43" t="n"/>
+      <c r="AM162" s="43" t="n"/>
       <c r="AN162" s="4" t="n"/>
-      <c r="AO162" s="48">
-        <f>BDP($B$162,"BEST_SALES","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AP162" s="43">
-        <f>BDP($B$162,"BEST_SALES","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AQ162" s="43">
-        <f>BDP($B$162,"BEST_SALES","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AR162" s="43">
-        <f>BDP($B$162,"BEST_SALES","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AS162" s="43">
-        <f>BDP($B$162,"BEST_SALES","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AO162" s="48" t="n"/>
+      <c r="AP162" s="43" t="n"/>
+      <c r="AQ162" s="43" t="n"/>
+      <c r="AR162" s="43" t="n"/>
+      <c r="AS162" s="43" t="n"/>
       <c r="AT162" s="4" t="n"/>
-      <c r="AU162" s="48">
-        <f>BDP($B$162,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","24Y")</f>
-        <v/>
-      </c>
-      <c r="AV162" s="43">
-        <f>BDP($B$162,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","25Y")</f>
-        <v/>
-      </c>
-      <c r="AW162" s="43">
-        <f>BDP($B$162,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","26Y")</f>
-        <v/>
-      </c>
-      <c r="AX162" s="43">
-        <f>BDP($B$162,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","27Y")</f>
-        <v/>
-      </c>
-      <c r="AY162" s="43">
-        <f>BDP($B$162,"BEST_EBIT","BEST_FPERIOD_OVERRIDE","28Y")</f>
-        <v/>
-      </c>
+      <c r="AU162" s="48" t="n"/>
+      <c r="AV162" s="43" t="n"/>
+      <c r="AW162" s="43" t="n"/>
+      <c r="AX162" s="43" t="n"/>
+      <c r="AY162" s="43" t="n"/>
       <c r="AZ162" s="4" t="n"/>
       <c r="BA162" s="1">
         <f>C162+BD162</f>
@@ -32081,10 +31139,7 @@
         <f>C162</f>
         <v/>
       </c>
-      <c r="BD162" s="43">
-        <f>BDP($B$162,"TRAIL_12M_EBITDA")</f>
-        <v/>
-      </c>
+      <c r="BD162" s="43" t="n"/>
       <c r="BE162" s="4" t="n"/>
       <c r="BF162" s="1" t="n"/>
       <c r="BG162" s="1" t="n"/>

</xml_diff>